<commit_message>
Completa pesos del catálogo Michelin
</commit_message>
<xml_diff>
--- a/outputs/catalogacion_vtex_michelin_2026-08-20/catalogacion_vtex_michelin_40_productos.xlsx
+++ b/outputs/catalogacion_vtex_michelin_2026-08-20/catalogacion_vtex_michelin_40_productos.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products 1" sheetId="1" r:id="R1f01abd584924f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products 1" sheetId="1" r:id="R0d417e28d01f4ace"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,6 +50,46 @@
     <x:author>tc={24CE852C-E8F0-2F8D-4510-0D4E2A5C3024}</x:author>
     <x:author>tc={45AB98E4-82EC-9D2B-66C8-7D90330187C6}</x:author>
     <x:author>tc={B3E6ED9A-FA7F-883F-FDCB-5D23E7A162DD}</x:author>
+    <x:author>tc={E167F516-8655-2415-0CA5-DBD87D9B7922}</x:author>
+    <x:author>tc={68947793-FA54-B749-ECED-1BA6A63A8FF6}</x:author>
+    <x:author>tc={BD12B8A3-D951-1D43-9160-66F7107BB1CD}</x:author>
+    <x:author>tc={C6215A16-C347-DD2B-45CF-1CA03767587E}</x:author>
+    <x:author>tc={FA4A5CDE-BDCF-D44A-98DE-441F63E256CE}</x:author>
+    <x:author>tc={CF7A5E8F-5AF4-5639-0187-555C1E505936}</x:author>
+    <x:author>tc={5AC9B3E0-DEB2-26C9-3E26-A37615693F29}</x:author>
+    <x:author>tc={6F2E39A5-44C4-FB7F-0D91-143C0A8BC52E}</x:author>
+    <x:author>tc={194F1AF5-A6B2-5877-2621-D151D21BA754}</x:author>
+    <x:author>tc={0A268E14-0FC5-8F02-203A-B810DEDF84AE}</x:author>
+    <x:author>tc={2DC8297A-991C-03A0-9D8C-DDAAF3CB23E9}</x:author>
+    <x:author>tc={03D8471C-1189-6E88-C75B-9AA99C67EB31}</x:author>
+    <x:author>tc={5FABA5A4-CCD8-210D-6F92-0C5D49D28C5B}</x:author>
+    <x:author>tc={46CC3662-14D9-5CCB-F410-034058840F6A}</x:author>
+    <x:author>tc={93F3DBE3-55C8-71AC-A181-524D2663E7EE}</x:author>
+    <x:author>tc={D6830E59-FAE9-AFE0-AA70-C4D60FD00CC4}</x:author>
+    <x:author>tc={CCA47167-1A8B-6080-5D9F-BAE45D34DD30}</x:author>
+    <x:author>tc={88371FA9-32D3-263C-9E5C-52509411B5ED}</x:author>
+    <x:author>tc={F0CDB466-5C68-0C06-A452-F2ED267605D6}</x:author>
+    <x:author>tc={EA83A53E-5868-EC32-E983-9764ED735AB4}</x:author>
+    <x:author>tc={B26A50CD-01CD-A80F-8D77-1D7AAA076DCD}</x:author>
+    <x:author>tc={356960CB-61AD-1DD2-E537-82E1115023A5}</x:author>
+    <x:author>tc={1E75472A-03FE-20EF-21D5-15581B52E5CE}</x:author>
+    <x:author>tc={BA6F2846-AEDC-231C-71AB-CC0826E7534B}</x:author>
+    <x:author>tc={47DF5790-AFB4-6BCB-D339-6C1B32733E7D}</x:author>
+    <x:author>tc={BEB2D71F-DFEF-9924-A228-E9A54CD4CE78}</x:author>
+    <x:author>tc={0EE3E580-C636-B928-D43E-6362C0E16F9F}</x:author>
+    <x:author>tc={66E1EB90-EAAF-FFCC-771D-590C2B725251}</x:author>
+    <x:author>tc={CE2C4E52-BEDE-2CE9-20F8-DCAF609A86BD}</x:author>
+    <x:author>tc={34A9219D-2384-2488-0AC0-523BE69C0F56}</x:author>
+    <x:author>tc={DDA562CD-F032-8CF0-BD23-5DB637F70B9E}</x:author>
+    <x:author>tc={0126FC1D-55FC-0E9C-BF18-2FFB6775EF94}</x:author>
+    <x:author>tc={1F9AA3BC-0175-4EC2-28BE-085C18659D1B}</x:author>
+    <x:author>tc={B246CCE9-7CCC-E623-A2C0-8063D1D13B02}</x:author>
+    <x:author>tc={3238B280-B158-1E33-1EA6-DE07AF181089}</x:author>
+    <x:author>tc={B60A2536-8AAE-36A1-74E5-414CE3D70BDF}</x:author>
+    <x:author>tc={BB5E2BB0-412E-CE3C-6200-F7C5A481A36C}</x:author>
+    <x:author>tc={04AE7A4E-27DE-AD60-A733-2ED905405872}</x:author>
+    <x:author>tc={D95005C5-A5D6-153D-033D-2885285C88B2}</x:author>
+    <x:author>tc={8FB2744A-8CE0-1DCD-4A44-9EA012A1957E}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B3" authorId="0">
@@ -449,6 +489,406 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Fuente de modelo: no se encontró ficha oficial específica vigente. Control: no activar automáticamente hasta validar categoría, marcación, imagen, EAN y datos logísticos cuando corresponda.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF3" authorId="40">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.300 g. Estimado por equivalencia: Michelin de altas prestaciones 285/30 R18; validar peso de la referencia N3. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF4" authorId="41">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.200 g. Estimado por equivalencia: Michelin turismo 215/55 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF5" authorId="42">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 20.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV de gran diámetro (315/35 R22); validar peso de la referencia ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF6" authorId="43">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 12.600 g. Estimado por equivalencia: Michelin Pilot Sport EV 235/55 R20 (13,3 kg) ajustado a R19; validar referencia Acoustic. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF7" authorId="44">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.700 g. Estimado por equivalencia: Michelin turismo 255/45 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF8" authorId="45">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 13.890 g. Peso de referencia exacta Michelin Agilis Alpin 205/75 R16C 110/108R: 13,89 kg. Fuente: https://reifen.auto.check24.de/ul/transporter-winterreifen/michelin-agilis-alpin-205-75r16c-110-108r-57174?cid=0&amp;trtid=31747819-0cdf-4c81-9844-4226d279583f El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF9" authorId="46">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 14.800 g. Estimado por equivalencia: Michelin Pilot Sport 4 de altas prestaciones 295/40 R19; validar marcación ND0. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF10" authorId="47">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 12.100 g. Estimado por equivalencia: Michelin turismo 235/55 R19; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF11" authorId="48">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 17.800 g. Estimado por equivalencia: Michelin Primacy SUV+ 285/60 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF12" authorId="49">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.800 g. Estimado por equivalencia: Michelin Pilot Sport 5 275/35 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF13" authorId="50">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 9.200 g. Estimado por equivalencia: Michelin turismo 215/60 R16; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF14" authorId="51">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 15.800 g. Estimado por equivalencia: Michelin de altas prestaciones 285/40 R20; validar modelo Pilot Sport 5S y marcación *. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF15" authorId="52">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 14.970 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 315/35 R20 (32-33 lb según Tire Rack); validar marcación K1. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF16" authorId="53">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 12.200 g. Estimado por equivalencia: Michelin e.Primacy 245/40 R20; validar marcación Acoustic. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF17" authorId="54">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.700 g. Estimado por equivalencia: Michelin turismo 215/65 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF18" authorId="55">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 13.200 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 235/55 R19; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF19" authorId="56">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.400 g. Estimado por equivalencia: Michelin Primacy 3 run flat 225/45 R17; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF20" authorId="57">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.700 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 235/40 R20; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF21" authorId="58">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 13.300 g. Peso de referencia exacta Michelin Pilot Sport EV 235/55 R20 105Y: 13,3 kg. Fuente: https://ecomplex.ro/produs/anvelopa-vara-michelin-pilot-sport-ev-235-55r20-lomi-105y-psevn-aderenta-b-consum-b/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF22" authorId="59">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 13.600 g. Peso de referencia exacta Michelin Pilot Sport Cup 2 315/30 R20 104Y: aprox. 13,6 kg (30 lb). Fuente: https://www.tirerack.com/tires/tires.jsp?partnum=13YR0PSC2XL&amp;sidewall=Blackwall&amp;tab=Sizes&amp;tireMake=Michelin&amp;tireModel=Pilot+Sport+Cup+2 El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF23" authorId="60">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 15.300 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 275/40 R20 run flat; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF24" authorId="61">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.500 g. Estimado por equivalencia: Michelin turismo 225/55 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF25" authorId="62">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 25.000 g. Estimado por equivalencia: neumático LT 285/70 R17 Load Range E 10 telas; validar peso de la referencia X LT A/S 2. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF26" authorId="63">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 3.680 g. Peso de referencia comparable Michelin Pilot Street 110/70-17 54S: 3,68 kg. Fuente: https://mmr-moto.ro/anvelopa-michelin-110-70-17-tl-tt-54s-pilot-street/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF27" authorId="64">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 17.800 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 275/40 R22 run flat; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF28" authorId="65">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 14.100 g. Peso de referencia exacta Michelin Pilot Sport 4 S 325/25 R20 101Y: aprox. 14,1 kg (31 lb). Fuente: https://www.tirerack.com/tires/tires.jsp?partnum=225YR0PS4SXL&amp;tireMake=Michelin&amp;tireModel=Pilot+Sport+4S El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF29" authorId="66">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.200 g. Peso de referencia exacta Michelin X-Ice Snow 225/45 R17 94H: aprox. 10,2 kg. Fuente: https://www.707.lv/automasinai/riepas/ziemas-riepas/225-45r17-michelin-x-ice-snow-94h-xl-rp-friction-cea69-3pmsf-icegrip-lv/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF30" authorId="67">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.900 g. Estimado por equivalencia: Michelin X-Ice Snow+ 215/65 R16, 24 lb (10,9 kg). Fuente comparable: https://www.tirerack.com/tires/Specifications.pdf?make=Michelin&amp;model=X-Ice+Snow%2B El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF31" authorId="68">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.600 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 265/30 R19; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF32" authorId="69">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.200 g. Estimado por equivalencia: Michelin de altas prestaciones 225/45 R17; validar marcación N3. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF33" authorId="70">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 13.300 g. Peso de referencia exacta por misma medida Michelin Pilot Sport EV 235/55 R20 105Y: 13,3 kg. Fuente: https://ecomplex.ro/produs/anvelopa-vara-michelin-pilot-sport-ev-235-55r20-lomi-105y-psevn-aderenta-b-consum-b/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF34" authorId="71">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 9.600 g. Estimado por equivalencia: Michelin Primacy 3 run flat 205/55 R16; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF35" authorId="72">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 16.500 g. Estimado por equivalencia: Michelin Primacy SUV+ 265/65 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF36" authorId="73">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 10.200 g. Estimado por equivalencia: Michelin Pilot Sport 5 245/45 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF37" authorId="74">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 11.400 g. Estimado por equivalencia: Michelin Pilot Sport 4 run flat 225/45 R19; validar tecnología EMT. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF38" authorId="75">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 9.200 g. Estimado por equivalencia: Michelin Primacy 5 215/55 R16; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF39" authorId="76">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 17.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 285/50 R20; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF40" authorId="77">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 9.600 g. Estimado por equivalencia: Michelin Primacy 5 235/45 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF41" authorId="78">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 19.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 295/40 R22; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+    <x:comment ref="AF42" authorId="79">
+      <x:text>
+        <x:r>
+          <x:t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Peso cargado: 400 g. Estimado por equivalencia: contenido de 330 ml más envase; validar peso bruto real con proveedor. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -462,9 +902,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0.00"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -502,7 +943,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -530,6 +971,9 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -540,6 +984,7 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
   <xltc:person displayName="Joaco" id="{7F16A6FE-E501-4086-8AFA-261888E44125}"/>
+  <xltc:person displayName="Joaco" id="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}"/>
 </xltc:personList>
 </file>
 
@@ -914,6 +1359,126 @@
   <xltc:threadedComment ref="B42" dT="2026-08-20T15:19:32.318" personId="{7F16A6FE-E501-4086-8AFA-261888E44125}" id="{B3E6ED9A-FA7F-883F-FDCB-5D23E7A162DD}">
     <xltc:text>Fuente de modelo: no se encontró ficha oficial específica vigente. Control: no activar automáticamente hasta validar categoría, marcación, imagen, EAN y datos logísticos cuando corresponda.</xltc:text>
   </xltc:threadedComment>
+  <xltc:threadedComment ref="AF3" dT="2026-08-20T16:32:11.082" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{E167F516-8655-2415-0CA5-DBD87D9B7922}">
+    <xltc:text>Peso cargado: 11.300 g. Estimado por equivalencia: Michelin de altas prestaciones 285/30 R18; validar peso de la referencia N3. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF4" dT="2026-08-20T16:32:11.092" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{68947793-FA54-B749-ECED-1BA6A63A8FF6}">
+    <xltc:text>Peso cargado: 11.200 g. Estimado por equivalencia: Michelin turismo 215/55 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF5" dT="2026-08-20T16:32:11.093" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{BD12B8A3-D951-1D43-9160-66F7107BB1CD}">
+    <xltc:text>Peso cargado: 20.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV de gran diámetro (315/35 R22); validar peso de la referencia ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF6" dT="2026-08-20T16:32:11.093" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{C6215A16-C347-DD2B-45CF-1CA03767587E}">
+    <xltc:text>Peso cargado: 12.600 g. Estimado por equivalencia: Michelin Pilot Sport EV 235/55 R20 (13,3 kg) ajustado a R19; validar referencia Acoustic. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF7" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{FA4A5CDE-BDCF-D44A-98DE-441F63E256CE}">
+    <xltc:text>Peso cargado: 11.700 g. Estimado por equivalencia: Michelin turismo 255/45 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF8" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{CF7A5E8F-5AF4-5639-0187-555C1E505936}">
+    <xltc:text>Peso cargado: 13.890 g. Peso de referencia exacta Michelin Agilis Alpin 205/75 R16C 110/108R: 13,89 kg. Fuente: https://reifen.auto.check24.de/ul/transporter-winterreifen/michelin-agilis-alpin-205-75r16c-110-108r-57174?cid=0&amp;trtid=31747819-0cdf-4c81-9844-4226d279583f El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF9" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{5AC9B3E0-DEB2-26C9-3E26-A37615693F29}">
+    <xltc:text>Peso cargado: 14.800 g. Estimado por equivalencia: Michelin Pilot Sport 4 de altas prestaciones 295/40 R19; validar marcación ND0. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF10" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{6F2E39A5-44C4-FB7F-0D91-143C0A8BC52E}">
+    <xltc:text>Peso cargado: 12.100 g. Estimado por equivalencia: Michelin turismo 235/55 R19; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF11" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{194F1AF5-A6B2-5877-2621-D151D21BA754}">
+    <xltc:text>Peso cargado: 17.800 g. Estimado por equivalencia: Michelin Primacy SUV+ 285/60 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF12" dT="2026-08-20T16:32:11.094" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{0A268E14-0FC5-8F02-203A-B810DEDF84AE}">
+    <xltc:text>Peso cargado: 11.800 g. Estimado por equivalencia: Michelin Pilot Sport 5 275/35 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF13" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{2DC8297A-991C-03A0-9D8C-DDAAF3CB23E9}">
+    <xltc:text>Peso cargado: 9.200 g. Estimado por equivalencia: Michelin turismo 215/60 R16; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF14" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{03D8471C-1189-6E88-C75B-9AA99C67EB31}">
+    <xltc:text>Peso cargado: 15.800 g. Estimado por equivalencia: Michelin de altas prestaciones 285/40 R20; validar modelo Pilot Sport 5S y marcación *. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF15" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{5FABA5A4-CCD8-210D-6F92-0C5D49D28C5B}">
+    <xltc:text>Peso cargado: 14.970 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 315/35 R20 (32-33 lb según Tire Rack); validar marcación K1. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF16" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{46CC3662-14D9-5CCB-F410-034058840F6A}">
+    <xltc:text>Peso cargado: 12.200 g. Estimado por equivalencia: Michelin e.Primacy 245/40 R20; validar marcación Acoustic. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF17" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{93F3DBE3-55C8-71AC-A181-524D2663E7EE}">
+    <xltc:text>Peso cargado: 10.700 g. Estimado por equivalencia: Michelin turismo 215/65 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF18" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{D6830E59-FAE9-AFE0-AA70-C4D60FD00CC4}">
+    <xltc:text>Peso cargado: 13.200 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 235/55 R19; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF19" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{CCA47167-1A8B-6080-5D9F-BAE45D34DD30}">
+    <xltc:text>Peso cargado: 10.400 g. Estimado por equivalencia: Michelin Primacy 3 run flat 225/45 R17; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF20" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{88371FA9-32D3-263C-9E5C-52509411B5ED}">
+    <xltc:text>Peso cargado: 11.700 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 235/40 R20; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF21" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{F0CDB466-5C68-0C06-A452-F2ED267605D6}">
+    <xltc:text>Peso cargado: 13.300 g. Peso de referencia exacta Michelin Pilot Sport EV 235/55 R20 105Y: 13,3 kg. Fuente: https://ecomplex.ro/produs/anvelopa-vara-michelin-pilot-sport-ev-235-55r20-lomi-105y-psevn-aderenta-b-consum-b/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF22" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{EA83A53E-5868-EC32-E983-9764ED735AB4}">
+    <xltc:text>Peso cargado: 13.600 g. Peso de referencia exacta Michelin Pilot Sport Cup 2 315/30 R20 104Y: aprox. 13,6 kg (30 lb). Fuente: https://www.tirerack.com/tires/tires.jsp?partnum=13YR0PSC2XL&amp;sidewall=Blackwall&amp;tab=Sizes&amp;tireMake=Michelin&amp;tireModel=Pilot+Sport+Cup+2 El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF23" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{B26A50CD-01CD-A80F-8D77-1D7AAA076DCD}">
+    <xltc:text>Peso cargado: 15.300 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 275/40 R20 run flat; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF24" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{356960CB-61AD-1DD2-E537-82E1115023A5}">
+    <xltc:text>Peso cargado: 10.500 g. Estimado por equivalencia: Michelin turismo 225/55 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF25" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{1E75472A-03FE-20EF-21D5-15581B52E5CE}">
+    <xltc:text>Peso cargado: 25.000 g. Estimado por equivalencia: neumático LT 285/70 R17 Load Range E 10 telas; validar peso de la referencia X LT A/S 2. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF26" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{BA6F2846-AEDC-231C-71AB-CC0826E7534B}">
+    <xltc:text>Peso cargado: 3.680 g. Peso de referencia comparable Michelin Pilot Street 110/70-17 54S: 3,68 kg. Fuente: https://mmr-moto.ro/anvelopa-michelin-110-70-17-tl-tt-54s-pilot-street/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF27" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{47DF5790-AFB4-6BCB-D339-6C1B32733E7D}">
+    <xltc:text>Peso cargado: 17.800 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 275/40 R22 run flat; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF28" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{BEB2D71F-DFEF-9924-A228-E9A54CD4CE78}">
+    <xltc:text>Peso cargado: 14.100 g. Peso de referencia exacta Michelin Pilot Sport 4 S 325/25 R20 101Y: aprox. 14,1 kg (31 lb). Fuente: https://www.tirerack.com/tires/tires.jsp?partnum=225YR0PS4SXL&amp;tireMake=Michelin&amp;tireModel=Pilot+Sport+4S El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF29" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{0EE3E580-C636-B928-D43E-6362C0E16F9F}">
+    <xltc:text>Peso cargado: 10.200 g. Peso de referencia exacta Michelin X-Ice Snow 225/45 R17 94H: aprox. 10,2 kg. Fuente: https://www.707.lv/automasinai/riepas/ziemas-riepas/225-45r17-michelin-x-ice-snow-94h-xl-rp-friction-cea69-3pmsf-icegrip-lv/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF30" dT="2026-08-20T16:32:11.095" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{66E1EB90-EAAF-FFCC-771D-590C2B725251}">
+    <xltc:text>Peso cargado: 10.900 g. Estimado por equivalencia: Michelin X-Ice Snow+ 215/65 R16, 24 lb (10,9 kg). Fuente comparable: https://www.tirerack.com/tires/Specifications.pdf?make=Michelin&amp;model=X-Ice+Snow%2B El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF31" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{CE2C4E52-BEDE-2CE9-20F8-DCAF609A86BD}">
+    <xltc:text>Peso cargado: 11.600 g. Estimado por equivalencia: Michelin Pilot Sport 4 S 265/30 R19; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF32" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{34A9219D-2384-2488-0AC0-523BE69C0F56}">
+    <xltc:text>Peso cargado: 10.200 g. Estimado por equivalencia: Michelin de altas prestaciones 225/45 R17; validar marcación N3. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF33" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{DDA562CD-F032-8CF0-BD23-5DB637F70B9E}">
+    <xltc:text>Peso cargado: 13.300 g. Peso de referencia exacta por misma medida Michelin Pilot Sport EV 235/55 R20 105Y: 13,3 kg. Fuente: https://ecomplex.ro/produs/anvelopa-vara-michelin-pilot-sport-ev-235-55r20-lomi-105y-psevn-aderenta-b-consum-b/ El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF34" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{0126FC1D-55FC-0E9C-BF18-2FFB6775EF94}">
+    <xltc:text>Peso cargado: 9.600 g. Estimado por equivalencia: Michelin Primacy 3 run flat 205/55 R16; validar tecnología ZP. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF35" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{1F9AA3BC-0175-4EC2-28BE-085C18659D1B}">
+    <xltc:text>Peso cargado: 16.500 g. Estimado por equivalencia: Michelin Primacy SUV+ 265/65 R18; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF36" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{B246CCE9-7CCC-E623-A2C0-8063D1D13B02}">
+    <xltc:text>Peso cargado: 10.200 g. Estimado por equivalencia: Michelin Pilot Sport 5 245/45 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF37" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{3238B280-B158-1E33-1EA6-DE07AF181089}">
+    <xltc:text>Peso cargado: 11.400 g. Estimado por equivalencia: Michelin Pilot Sport 4 run flat 225/45 R19; validar tecnología EMT. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF38" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{B60A2536-8AAE-36A1-74E5-414CE3D70BDF}">
+    <xltc:text>Peso cargado: 9.200 g. Estimado por equivalencia: Michelin Primacy 5 215/55 R16; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF39" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{BB5E2BB0-412E-CE3C-6200-F7C5A481A36C}">
+    <xltc:text>Peso cargado: 17.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 285/50 R20; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF40" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{04AE7A4E-27DE-AD60-A733-2ED905405872}">
+    <xltc:text>Peso cargado: 9.600 g. Estimado por equivalencia: Michelin Primacy 5 235/45 R17; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF41" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{D95005C5-A5D6-153D-033D-2885285C88B2}">
+    <xltc:text>Peso cargado: 19.500 g. Estimado por equivalencia: Michelin Pilot Sport 4 SUV 295/40 R22; validar peso de la referencia exacta. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="AF42" dT="2026-08-20T16:32:11.096" personId="{F5601A89-5FA7-4A1D-BBB5-ABE82B4319BA}" id="{8FB2744A-8CE0-1DCD-4A44-9EA012A1957E}">
+    <xltc:text>Peso cargado: 400 g. Estimado por equivalencia: contenido de 330 ml más envase; validar peso bruto real con proveedor. El peso de paquete se iguala al peso de cubierta como valor logístico provisorio; validar embalaje final.</xltc:text>
+  </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>
 
@@ -1252,7 +1817,9 @@
       <x:c r="AE3" s="4" t="str">
         <x:v>40653</x:v>
       </x:c>
-      <x:c r="AF3" s="5"/>
+      <x:c r="AF3" s="11" t="n">
+        <x:v>11300</x:v>
+      </x:c>
       <x:c r="AG3" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -1262,7 +1829,9 @@
       <x:c r="AI3" s="5" t="n">
         <x:v>62.82</x:v>
       </x:c>
-      <x:c r="AJ3" s="5"/>
+      <x:c r="AJ3" s="11" t="n">
+        <x:v>11300</x:v>
+      </x:c>
       <x:c r="AK3" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -1360,7 +1929,9 @@
       <x:c r="AE4" s="4" t="str">
         <x:v>44495</x:v>
       </x:c>
-      <x:c r="AF4" s="5"/>
+      <x:c r="AF4" s="11" t="n">
+        <x:v>11200</x:v>
+      </x:c>
       <x:c r="AG4" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -1370,7 +1941,9 @@
       <x:c r="AI4" s="5" t="n">
         <x:v>69.37</x:v>
       </x:c>
-      <x:c r="AJ4" s="5"/>
+      <x:c r="AJ4" s="11" t="n">
+        <x:v>11200</x:v>
+      </x:c>
       <x:c r="AK4" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -1468,7 +2041,9 @@
       <x:c r="AE5" s="4" t="str">
         <x:v>61438</x:v>
       </x:c>
-      <x:c r="AF5" s="5"/>
+      <x:c r="AF5" s="11" t="n">
+        <x:v>20500</x:v>
+      </x:c>
       <x:c r="AG5" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -1478,7 +2053,9 @@
       <x:c r="AI5" s="5" t="n">
         <x:v>77.93</x:v>
       </x:c>
-      <x:c r="AJ5" s="5"/>
+      <x:c r="AJ5" s="11" t="n">
+        <x:v>20500</x:v>
+      </x:c>
       <x:c r="AK5" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -1576,7 +2153,9 @@
       <x:c r="AE6" s="4" t="str">
         <x:v>102099</x:v>
       </x:c>
-      <x:c r="AF6" s="5"/>
+      <x:c r="AF6" s="11" t="n">
+        <x:v>12600</x:v>
+      </x:c>
       <x:c r="AG6" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -1586,7 +2165,9 @@
       <x:c r="AI6" s="5" t="n">
         <x:v>74.11</x:v>
       </x:c>
-      <x:c r="AJ6" s="5"/>
+      <x:c r="AJ6" s="11" t="n">
+        <x:v>12600</x:v>
+      </x:c>
       <x:c r="AK6" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -1684,7 +2265,9 @@
       <x:c r="AE7" s="4" t="str">
         <x:v>121427</x:v>
       </x:c>
-      <x:c r="AF7" s="5"/>
+      <x:c r="AF7" s="11" t="n">
+        <x:v>11700</x:v>
+      </x:c>
       <x:c r="AG7" s="5" t="n">
         <x:v>25.5</x:v>
       </x:c>
@@ -1694,7 +2277,9 @@
       <x:c r="AI7" s="5" t="n">
         <x:v>68.67</x:v>
       </x:c>
-      <x:c r="AJ7" s="5"/>
+      <x:c r="AJ7" s="11" t="n">
+        <x:v>11700</x:v>
+      </x:c>
       <x:c r="AK7" s="5" t="n">
         <x:v>25.5</x:v>
       </x:c>
@@ -1788,7 +2373,9 @@
       <x:c r="AE8" s="4" t="str">
         <x:v>159386</x:v>
       </x:c>
-      <x:c r="AF8" s="5"/>
+      <x:c r="AF8" s="11" t="n">
+        <x:v>13890</x:v>
+      </x:c>
       <x:c r="AG8" s="5" t="n">
         <x:v>20.5</x:v>
       </x:c>
@@ -1798,7 +2385,9 @@
       <x:c r="AI8" s="5" t="n">
         <x:v>71.39</x:v>
       </x:c>
-      <x:c r="AJ8" s="5"/>
+      <x:c r="AJ8" s="11" t="n">
+        <x:v>13890</x:v>
+      </x:c>
       <x:c r="AK8" s="5" t="n">
         <x:v>20.5</x:v>
       </x:c>
@@ -1896,7 +2485,9 @@
       <x:c r="AE9" s="4" t="str">
         <x:v>179561</x:v>
       </x:c>
-      <x:c r="AF9" s="5"/>
+      <x:c r="AF9" s="11" t="n">
+        <x:v>14800</x:v>
+      </x:c>
       <x:c r="AG9" s="5" t="n">
         <x:v>29.5</x:v>
       </x:c>
@@ -1906,7 +2497,9 @@
       <x:c r="AI9" s="5" t="n">
         <x:v>71.86</x:v>
       </x:c>
-      <x:c r="AJ9" s="5"/>
+      <x:c r="AJ9" s="11" t="n">
+        <x:v>14800</x:v>
+      </x:c>
       <x:c r="AK9" s="5" t="n">
         <x:v>29.5</x:v>
       </x:c>
@@ -2004,7 +2597,9 @@
       <x:c r="AE10" s="4" t="str">
         <x:v>192003</x:v>
       </x:c>
-      <x:c r="AF10" s="5"/>
+      <x:c r="AF10" s="11" t="n">
+        <x:v>12100</x:v>
+      </x:c>
       <x:c r="AG10" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -2014,7 +2609,9 @@
       <x:c r="AI10" s="5" t="n">
         <x:v>74.11</x:v>
       </x:c>
-      <x:c r="AJ10" s="5"/>
+      <x:c r="AJ10" s="11" t="n">
+        <x:v>12100</x:v>
+      </x:c>
       <x:c r="AK10" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -2112,7 +2709,9 @@
       <x:c r="AE11" s="4" t="str">
         <x:v>234050</x:v>
       </x:c>
-      <x:c r="AF11" s="5"/>
+      <x:c r="AF11" s="11" t="n">
+        <x:v>17800</x:v>
+      </x:c>
       <x:c r="AG11" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -2122,7 +2721,9 @@
       <x:c r="AI11" s="5" t="n">
         <x:v>79.92</x:v>
       </x:c>
-      <x:c r="AJ11" s="5"/>
+      <x:c r="AJ11" s="11" t="n">
+        <x:v>17800</x:v>
+      </x:c>
       <x:c r="AK11" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -2220,7 +2821,9 @@
       <x:c r="AE12" s="4" t="str">
         <x:v>269665</x:v>
       </x:c>
-      <x:c r="AF12" s="5"/>
+      <x:c r="AF12" s="11" t="n">
+        <x:v>11800</x:v>
+      </x:c>
       <x:c r="AG12" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -2230,7 +2833,9 @@
       <x:c r="AI12" s="5" t="n">
         <x:v>64.97</x:v>
       </x:c>
-      <x:c r="AJ12" s="5"/>
+      <x:c r="AJ12" s="11" t="n">
+        <x:v>11800</x:v>
+      </x:c>
       <x:c r="AK12" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -2328,7 +2933,9 @@
       <x:c r="AE13" s="4" t="str">
         <x:v>330554</x:v>
       </x:c>
-      <x:c r="AF13" s="5"/>
+      <x:c r="AF13" s="11" t="n">
+        <x:v>9200</x:v>
+      </x:c>
       <x:c r="AG13" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -2338,7 +2945,9 @@
       <x:c r="AI13" s="5" t="n">
         <x:v>66.44</x:v>
       </x:c>
-      <x:c r="AJ13" s="5"/>
+      <x:c r="AJ13" s="11" t="n">
+        <x:v>9200</x:v>
+      </x:c>
       <x:c r="AK13" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -2434,7 +3043,9 @@
       <x:c r="AE14" s="4" t="str">
         <x:v>331319</x:v>
       </x:c>
-      <x:c r="AF14" s="5"/>
+      <x:c r="AF14" s="11" t="n">
+        <x:v>15800</x:v>
+      </x:c>
       <x:c r="AG14" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -2444,7 +3055,9 @@
       <x:c r="AI14" s="5" t="n">
         <x:v>73.6</x:v>
       </x:c>
-      <x:c r="AJ14" s="5"/>
+      <x:c r="AJ14" s="11" t="n">
+        <x:v>15800</x:v>
+      </x:c>
       <x:c r="AK14" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -2542,7 +3155,9 @@
       <x:c r="AE15" s="4" t="str">
         <x:v>341013</x:v>
       </x:c>
-      <x:c r="AF15" s="5"/>
+      <x:c r="AF15" s="11" t="n">
+        <x:v>14970</x:v>
+      </x:c>
       <x:c r="AG15" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -2552,7 +3167,9 @@
       <x:c r="AI15" s="5" t="n">
         <x:v>72.85</x:v>
       </x:c>
-      <x:c r="AJ15" s="5"/>
+      <x:c r="AJ15" s="11" t="n">
+        <x:v>14970</x:v>
+      </x:c>
       <x:c r="AK15" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -2650,7 +3267,9 @@
       <x:c r="AE16" s="4" t="str">
         <x:v>409706</x:v>
       </x:c>
-      <x:c r="AF16" s="5"/>
+      <x:c r="AF16" s="11" t="n">
+        <x:v>12200</x:v>
+      </x:c>
       <x:c r="AG16" s="5" t="n">
         <x:v>24.5</x:v>
       </x:c>
@@ -2660,7 +3279,9 @@
       <x:c r="AI16" s="5" t="n">
         <x:v>70.4</x:v>
       </x:c>
-      <x:c r="AJ16" s="5"/>
+      <x:c r="AJ16" s="11" t="n">
+        <x:v>12200</x:v>
+      </x:c>
       <x:c r="AK16" s="5" t="n">
         <x:v>24.5</x:v>
       </x:c>
@@ -2758,7 +3379,9 @@
       <x:c r="AE17" s="4" t="str">
         <x:v>443497</x:v>
       </x:c>
-      <x:c r="AF17" s="5"/>
+      <x:c r="AF17" s="11" t="n">
+        <x:v>10700</x:v>
+      </x:c>
       <x:c r="AG17" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -2768,7 +3391,9 @@
       <x:c r="AI17" s="5" t="n">
         <x:v>71.13</x:v>
       </x:c>
-      <x:c r="AJ17" s="5"/>
+      <x:c r="AJ17" s="11" t="n">
+        <x:v>10700</x:v>
+      </x:c>
       <x:c r="AK17" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -2866,7 +3491,9 @@
       <x:c r="AE18" s="4" t="str">
         <x:v>459601</x:v>
       </x:c>
-      <x:c r="AF18" s="5"/>
+      <x:c r="AF18" s="11" t="n">
+        <x:v>13200</x:v>
+      </x:c>
       <x:c r="AG18" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -2876,7 +3503,9 @@
       <x:c r="AI18" s="5" t="n">
         <x:v>74.11</x:v>
       </x:c>
-      <x:c r="AJ18" s="5"/>
+      <x:c r="AJ18" s="11" t="n">
+        <x:v>13200</x:v>
+      </x:c>
       <x:c r="AK18" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -2974,7 +3603,9 @@
       <x:c r="AE19" s="4" t="str">
         <x:v>507226</x:v>
       </x:c>
-      <x:c r="AF19" s="5"/>
+      <x:c r="AF19" s="11" t="n">
+        <x:v>10400</x:v>
+      </x:c>
       <x:c r="AG19" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -2984,7 +3615,9 @@
       <x:c r="AI19" s="5" t="n">
         <x:v>63.43</x:v>
       </x:c>
-      <x:c r="AJ19" s="5"/>
+      <x:c r="AJ19" s="11" t="n">
+        <x:v>10400</x:v>
+      </x:c>
       <x:c r="AK19" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -3082,7 +3715,9 @@
       <x:c r="AE20" s="4" t="str">
         <x:v>524294</x:v>
       </x:c>
-      <x:c r="AF20" s="5"/>
+      <x:c r="AF20" s="11" t="n">
+        <x:v>11700</x:v>
+      </x:c>
       <x:c r="AG20" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -3092,7 +3727,9 @@
       <x:c r="AI20" s="5" t="n">
         <x:v>69.6</x:v>
       </x:c>
-      <x:c r="AJ20" s="5"/>
+      <x:c r="AJ20" s="11" t="n">
+        <x:v>11700</x:v>
+      </x:c>
       <x:c r="AK20" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -3190,7 +3827,9 @@
       <x:c r="AE21" s="4" t="str">
         <x:v>546825</x:v>
       </x:c>
-      <x:c r="AF21" s="5"/>
+      <x:c r="AF21" s="11" t="n">
+        <x:v>13300</x:v>
+      </x:c>
       <x:c r="AG21" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -3200,7 +3839,9 @@
       <x:c r="AI21" s="5" t="n">
         <x:v>76.65</x:v>
       </x:c>
-      <x:c r="AJ21" s="5"/>
+      <x:c r="AJ21" s="11" t="n">
+        <x:v>13300</x:v>
+      </x:c>
       <x:c r="AK21" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -3298,7 +3939,9 @@
       <x:c r="AE22" s="4" t="str">
         <x:v>564253</x:v>
       </x:c>
-      <x:c r="AF22" s="5"/>
+      <x:c r="AF22" s="11" t="n">
+        <x:v>13600</x:v>
+      </x:c>
       <x:c r="AG22" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -3308,7 +3951,9 @@
       <x:c r="AI22" s="5" t="n">
         <x:v>69.7</x:v>
       </x:c>
-      <x:c r="AJ22" s="5"/>
+      <x:c r="AJ22" s="11" t="n">
+        <x:v>13600</x:v>
+      </x:c>
       <x:c r="AK22" s="5" t="n">
         <x:v>31.5</x:v>
       </x:c>
@@ -3406,7 +4051,9 @@
       <x:c r="AE23" s="4" t="str">
         <x:v>657707</x:v>
       </x:c>
-      <x:c r="AF23" s="5"/>
+      <x:c r="AF23" s="11" t="n">
+        <x:v>15300</x:v>
+      </x:c>
       <x:c r="AG23" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -3416,7 +4063,9 @@
       <x:c r="AI23" s="5" t="n">
         <x:v>72.8</x:v>
       </x:c>
-      <x:c r="AJ23" s="5"/>
+      <x:c r="AJ23" s="11" t="n">
+        <x:v>15300</x:v>
+      </x:c>
       <x:c r="AK23" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -3514,7 +4163,9 @@
       <x:c r="AE24" s="4" t="str">
         <x:v>696861</x:v>
       </x:c>
-      <x:c r="AF24" s="5"/>
+      <x:c r="AF24" s="11" t="n">
+        <x:v>10500</x:v>
+      </x:c>
       <x:c r="AG24" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -3524,7 +4175,9 @@
       <x:c r="AI24" s="5" t="n">
         <x:v>67.93</x:v>
       </x:c>
-      <x:c r="AJ24" s="5"/>
+      <x:c r="AJ24" s="11" t="n">
+        <x:v>10500</x:v>
+      </x:c>
       <x:c r="AK24" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -3622,7 +4275,9 @@
       <x:c r="AE25" s="4" t="str">
         <x:v>699744</x:v>
       </x:c>
-      <x:c r="AF25" s="5"/>
+      <x:c r="AF25" s="11" t="n">
+        <x:v>25000</x:v>
+      </x:c>
       <x:c r="AG25" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -3632,7 +4287,9 @@
       <x:c r="AI25" s="5" t="n">
         <x:v>83.08</x:v>
       </x:c>
-      <x:c r="AJ25" s="5"/>
+      <x:c r="AJ25" s="11" t="n">
+        <x:v>25000</x:v>
+      </x:c>
       <x:c r="AK25" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -3726,7 +4383,9 @@
       <x:c r="AE26" s="4" t="str">
         <x:v>718236</x:v>
       </x:c>
-      <x:c r="AF26" s="5"/>
+      <x:c r="AF26" s="11" t="n">
+        <x:v>3680</x:v>
+      </x:c>
       <x:c r="AG26" s="5" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -3736,7 +4395,9 @@
       <x:c r="AI26" s="5" t="n">
         <x:v>58.58</x:v>
       </x:c>
-      <x:c r="AJ26" s="5"/>
+      <x:c r="AJ26" s="11" t="n">
+        <x:v>3680</x:v>
+      </x:c>
       <x:c r="AK26" s="5" t="n">
         <x:v>11</x:v>
       </x:c>
@@ -3834,7 +4495,9 @@
       <x:c r="AE27" s="4" t="str">
         <x:v>747930</x:v>
       </x:c>
-      <x:c r="AF27" s="5"/>
+      <x:c r="AF27" s="11" t="n">
+        <x:v>17800</x:v>
+      </x:c>
       <x:c r="AG27" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -3844,7 +4507,9 @@
       <x:c r="AI27" s="5" t="n">
         <x:v>77.88</x:v>
       </x:c>
-      <x:c r="AJ27" s="5"/>
+      <x:c r="AJ27" s="11" t="n">
+        <x:v>17800</x:v>
+      </x:c>
       <x:c r="AK27" s="5" t="n">
         <x:v>27.5</x:v>
       </x:c>
@@ -3942,7 +4607,9 @@
       <x:c r="AE28" s="4" t="str">
         <x:v>748034</x:v>
       </x:c>
-      <x:c r="AF28" s="5"/>
+      <x:c r="AF28" s="11" t="n">
+        <x:v>14100</x:v>
+      </x:c>
       <x:c r="AG28" s="5" t="n">
         <x:v>32.5</x:v>
       </x:c>
@@ -3952,7 +4619,9 @@
       <x:c r="AI28" s="5" t="n">
         <x:v>67.05</x:v>
       </x:c>
-      <x:c r="AJ28" s="5"/>
+      <x:c r="AJ28" s="11" t="n">
+        <x:v>14100</x:v>
+      </x:c>
       <x:c r="AK28" s="5" t="n">
         <x:v>32.5</x:v>
       </x:c>
@@ -4050,7 +4719,9 @@
       <x:c r="AE29" s="4" t="str">
         <x:v>812083</x:v>
       </x:c>
-      <x:c r="AF29" s="5"/>
+      <x:c r="AF29" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AG29" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -4060,7 +4731,9 @@
       <x:c r="AI29" s="5" t="n">
         <x:v>63.43</x:v>
       </x:c>
-      <x:c r="AJ29" s="5"/>
+      <x:c r="AJ29" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AK29" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -4158,7 +4831,9 @@
       <x:c r="AE30" s="4" t="str">
         <x:v>812454</x:v>
       </x:c>
-      <x:c r="AF30" s="5"/>
+      <x:c r="AF30" s="11" t="n">
+        <x:v>10900</x:v>
+      </x:c>
       <x:c r="AG30" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -4168,7 +4843,9 @@
       <x:c r="AI30" s="5" t="n">
         <x:v>68.59</x:v>
       </x:c>
-      <x:c r="AJ30" s="5"/>
+      <x:c r="AJ30" s="11" t="n">
+        <x:v>10900</x:v>
+      </x:c>
       <x:c r="AK30" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -4266,7 +4943,9 @@
       <x:c r="AE31" s="4" t="str">
         <x:v>814204</x:v>
       </x:c>
-      <x:c r="AF31" s="5"/>
+      <x:c r="AF31" s="11" t="n">
+        <x:v>11600</x:v>
+      </x:c>
       <x:c r="AG31" s="5" t="n">
         <x:v>26.5</x:v>
       </x:c>
@@ -4276,7 +4955,9 @@
       <x:c r="AI31" s="5" t="n">
         <x:v>64.16</x:v>
       </x:c>
-      <x:c r="AJ31" s="5"/>
+      <x:c r="AJ31" s="11" t="n">
+        <x:v>11600</x:v>
+      </x:c>
       <x:c r="AK31" s="5" t="n">
         <x:v>26.5</x:v>
       </x:c>
@@ -4374,7 +5055,9 @@
       <x:c r="AE32" s="4" t="str">
         <x:v>823718</x:v>
       </x:c>
-      <x:c r="AF32" s="5"/>
+      <x:c r="AF32" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AG32" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -4384,7 +5067,9 @@
       <x:c r="AI32" s="5" t="n">
         <x:v>63.43</x:v>
       </x:c>
-      <x:c r="AJ32" s="5"/>
+      <x:c r="AJ32" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AK32" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -4482,7 +5167,9 @@
       <x:c r="AE33" s="4" t="str">
         <x:v>825359</x:v>
       </x:c>
-      <x:c r="AF33" s="5"/>
+      <x:c r="AF33" s="11" t="n">
+        <x:v>13300</x:v>
+      </x:c>
       <x:c r="AG33" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -4492,7 +5179,9 @@
       <x:c r="AI33" s="5" t="n">
         <x:v>76.65</x:v>
       </x:c>
-      <x:c r="AJ33" s="5"/>
+      <x:c r="AJ33" s="11" t="n">
+        <x:v>13300</x:v>
+      </x:c>
       <x:c r="AK33" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -4590,7 +5279,9 @@
       <x:c r="AE34" s="4" t="str">
         <x:v>871732</x:v>
       </x:c>
-      <x:c r="AF34" s="5"/>
+      <x:c r="AF34" s="11" t="n">
+        <x:v>9600</x:v>
+      </x:c>
       <x:c r="AG34" s="5" t="n">
         <x:v>20.5</x:v>
       </x:c>
@@ -4600,7 +5291,9 @@
       <x:c r="AI34" s="5" t="n">
         <x:v>63.19</x:v>
       </x:c>
-      <x:c r="AJ34" s="5"/>
+      <x:c r="AJ34" s="11" t="n">
+        <x:v>9600</x:v>
+      </x:c>
       <x:c r="AK34" s="5" t="n">
         <x:v>20.5</x:v>
       </x:c>
@@ -4698,7 +5391,9 @@
       <x:c r="AE35" s="4" t="str">
         <x:v>932908</x:v>
       </x:c>
-      <x:c r="AF35" s="5"/>
+      <x:c r="AF35" s="11" t="n">
+        <x:v>16500</x:v>
+      </x:c>
       <x:c r="AG35" s="5" t="n">
         <x:v>26.5</x:v>
       </x:c>
@@ -4708,7 +5403,9 @@
       <x:c r="AI35" s="5" t="n">
         <x:v>80.17</x:v>
       </x:c>
-      <x:c r="AJ35" s="5"/>
+      <x:c r="AJ35" s="11" t="n">
+        <x:v>16500</x:v>
+      </x:c>
       <x:c r="AK35" s="5" t="n">
         <x:v>26.5</x:v>
       </x:c>
@@ -4806,7 +5503,9 @@
       <x:c r="AE36" s="4" t="str">
         <x:v>951919</x:v>
       </x:c>
-      <x:c r="AF36" s="5"/>
+      <x:c r="AF36" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AG36" s="5" t="n">
         <x:v>24.5</x:v>
       </x:c>
@@ -4816,7 +5515,9 @@
       <x:c r="AI36" s="5" t="n">
         <x:v>65.23</x:v>
       </x:c>
-      <x:c r="AJ36" s="5"/>
+      <x:c r="AJ36" s="11" t="n">
+        <x:v>10200</x:v>
+      </x:c>
       <x:c r="AK36" s="5" t="n">
         <x:v>24.5</x:v>
       </x:c>
@@ -4914,7 +5615,9 @@
       <x:c r="AE37" s="4" t="str">
         <x:v>960559</x:v>
       </x:c>
-      <x:c r="AF37" s="5"/>
+      <x:c r="AF37" s="11" t="n">
+        <x:v>11400</x:v>
+      </x:c>
       <x:c r="AG37" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -4924,7 +5627,9 @@
       <x:c r="AI37" s="5" t="n">
         <x:v>68.51</x:v>
       </x:c>
-      <x:c r="AJ37" s="5"/>
+      <x:c r="AJ37" s="11" t="n">
+        <x:v>11400</x:v>
+      </x:c>
       <x:c r="AK37" s="5" t="n">
         <x:v>22.5</x:v>
       </x:c>
@@ -5022,7 +5727,9 @@
       <x:c r="AE38" s="4" t="str">
         <x:v>974855</x:v>
       </x:c>
-      <x:c r="AF38" s="5"/>
+      <x:c r="AF38" s="11" t="n">
+        <x:v>9200</x:v>
+      </x:c>
       <x:c r="AG38" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -5032,7 +5739,9 @@
       <x:c r="AI38" s="5" t="n">
         <x:v>64.29</x:v>
       </x:c>
-      <x:c r="AJ38" s="5"/>
+      <x:c r="AJ38" s="11" t="n">
+        <x:v>9200</x:v>
+      </x:c>
       <x:c r="AK38" s="5" t="n">
         <x:v>21.5</x:v>
       </x:c>
@@ -5130,7 +5839,9 @@
       <x:c r="AE39" s="4" t="str">
         <x:v>983867</x:v>
       </x:c>
-      <x:c r="AF39" s="5"/>
+      <x:c r="AF39" s="11" t="n">
+        <x:v>17500</x:v>
+      </x:c>
       <x:c r="AG39" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -5140,7 +5851,9 @@
       <x:c r="AI39" s="5" t="n">
         <x:v>79.3</x:v>
       </x:c>
-      <x:c r="AJ39" s="5"/>
+      <x:c r="AJ39" s="11" t="n">
+        <x:v>17500</x:v>
+      </x:c>
       <x:c r="AK39" s="5" t="n">
         <x:v>28.5</x:v>
       </x:c>
@@ -5238,7 +5951,9 @@
       <x:c r="AE40" s="4" t="str">
         <x:v>989426</x:v>
       </x:c>
-      <x:c r="AF40" s="5"/>
+      <x:c r="AF40" s="11" t="n">
+        <x:v>9600</x:v>
+      </x:c>
       <x:c r="AG40" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -5248,7 +5963,9 @@
       <x:c r="AI40" s="5" t="n">
         <x:v>64.33</x:v>
       </x:c>
-      <x:c r="AJ40" s="5"/>
+      <x:c r="AJ40" s="11" t="n">
+        <x:v>9600</x:v>
+      </x:c>
       <x:c r="AK40" s="5" t="n">
         <x:v>23.5</x:v>
       </x:c>
@@ -5346,7 +6063,9 @@
       <x:c r="AE41" s="4" t="str">
         <x:v>993345</x:v>
       </x:c>
-      <x:c r="AF41" s="5"/>
+      <x:c r="AF41" s="11" t="n">
+        <x:v>19500</x:v>
+      </x:c>
       <x:c r="AG41" s="5" t="n">
         <x:v>29.5</x:v>
       </x:c>
@@ -5356,7 +6075,9 @@
       <x:c r="AI41" s="5" t="n">
         <x:v>79.48</x:v>
       </x:c>
-      <x:c r="AJ41" s="5"/>
+      <x:c r="AJ41" s="11" t="n">
+        <x:v>19500</x:v>
+      </x:c>
       <x:c r="AK41" s="5" t="n">
         <x:v>29.5</x:v>
       </x:c>
@@ -5450,11 +6171,15 @@
       <x:c r="AE42" s="4" t="str">
         <x:v>RCVM-330</x:v>
       </x:c>
-      <x:c r="AF42" s="5"/>
+      <x:c r="AF42" s="11" t="n">
+        <x:v>400</x:v>
+      </x:c>
       <x:c r="AG42" s="5"/>
       <x:c r="AH42" s="5"/>
       <x:c r="AI42" s="5"/>
-      <x:c r="AJ42" s="5"/>
+      <x:c r="AJ42" s="11" t="n">
+        <x:v>400</x:v>
+      </x:c>
       <x:c r="AK42" s="5"/>
       <x:c r="AL42" s="5"/>
       <x:c r="AM42" s="5"/>
@@ -5476,9 +6201,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74c84f75aaba4332"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re085b2d1cb9747e9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3de4b9cf04ba402f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R224ce4c7333242ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>